<commit_message>
Restructure the game into Race for Life, Brand and Giving tabs
The budget chapter now lives on the Race for Life tab below the main
screen, the long-game chapter is renamed Brand, and the stage numbering,
VBA dispatcher, tests, room notes and README follow. The VBA stays core
Excel only so it runs on Excel for Mac as well as Windows.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFB7finRRwjLofP9hApkAo
</commit_message>
<xml_diff>
--- a/econometrics-game/CRUK_Econometrics_Game_v3_no_macros.xlsx
+++ b/econometrics-game/CRUK_Econometrics_Game_v3_no_macros.xlsx
@@ -7,17 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Play" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long game" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giving" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finish" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Words" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Under the bonnet" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="8" state="hidden" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room notes" sheetId="10" state="hidden" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="11" state="veryHidden" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Race for Life" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Brand" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giving" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finish" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Words" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Under the bonnet" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Room notes" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="10" state="veryHidden" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -314,6 +313,15 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BBC7D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="00BBC7D9"/>
       </top>
@@ -333,19 +341,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color rgb="00BBC7D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BBC7D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BBC7D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color rgb="00BBC7D9"/>
@@ -357,8 +352,12 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top/>
+      <right style="thin">
+        <color rgb="00BBC7D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBC7D9"/>
+      </top>
       <bottom style="thin">
         <color rgb="00BBC7D9"/>
       </bottom>
@@ -517,8 +516,8 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1522,7 +1521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:Z31"/>
+  <dimension ref="B2:Z55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1557,7 +1556,7 @@
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="1">
-        <f>"Chapter "&amp;INDEX(Steps!$B$2:$B$22,State!$B$1)&amp;"  ·  "&amp;INDEX(Steps!$C$2:$C$22,State!$B$1)</f>
+        <f>"Chapter "&amp;INDEX(Steps!$B$2:$B$23,State!$B$1)&amp;"  ·  "&amp;INDEX(Steps!$C$2:$C$23,State!$B$1)</f>
         <v/>
       </c>
       <c r="T2" s="2">
@@ -1594,14 +1593,14 @@
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="40" customHeight="1">
       <c r="B5" s="4">
-        <f>INDEX(Steps!$D$2:$D$22,State!$B$1)</f>
+        <f>INDEX(Steps!$D$2:$D$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="6" customHeight="1"/>
     <row r="7" ht="48" customHeight="1">
       <c r="B7" s="5">
-        <f>INDEX(Steps!$E$2:$E$22,State!$B$1)</f>
+        <f>INDEX(Steps!$E$2:$E$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -1628,7 +1627,7 @@
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="T11" s="8">
-        <f>IF(State!$B$33="dial",TEXT(State!$B$37,State!$B$45),IF(State!$B$33="quiz","A.   "&amp;INDEX(Steps!$O$2:$O$22,State!$B$1),IF(State!$B$33="dials5","TV:  "&amp;TEXT(State!$B$8,"0.0")&amp;" per £1,000",IF(State!$B$33="tests","Pattern explained",""))))</f>
+        <f>IF(State!$B$33="dial",TEXT(State!$B$37,State!$B$45),IF(State!$B$33="quiz","A.   "&amp;INDEX(Steps!$O$2:$O$23,State!$B$1),IF(State!$B$33="dials5","TV:  "&amp;TEXT(State!$B$8,"0.0")&amp;" per £1,000",IF(State!$B$33="tests","Pattern explained",""))))</f>
         <v/>
       </c>
       <c r="U11" s="9">
@@ -1688,7 +1687,7 @@
     </row>
     <row r="13" ht="26" customHeight="1">
       <c r="T13" s="8">
-        <f>IF(State!$B$33="quiz","B.   "&amp;INDEX(Steps!$P$2:$P$22,State!$B$1),IF(State!$B$33="dials5","Radio:  "&amp;TEXT(State!$B$10,"0.0")&amp;" per £1,000",IF(State!$B$33="tests","Predicts 2025","")))</f>
+        <f>IF(State!$B$33="quiz","B.   "&amp;INDEX(Steps!$P$2:$P$23,State!$B$1),IF(State!$B$33="dials5","Radio:  "&amp;TEXT(State!$B$10,"0.0")&amp;" per £1,000",IF(State!$B$33="tests","Predicts 2025","")))</f>
         <v/>
       </c>
       <c r="U13" s="9">
@@ -1748,7 +1747,7 @@
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="T15" s="8">
-        <f>IF(State!$B$33="quiz","C.   "&amp;INDEX(Steps!$Q$2:$Q$22,State!$B$1),IF(State!$B$33="dials5","Digital and social:  "&amp;TEXT(State!$B$12,"0.0")&amp;" per £1,000",""))</f>
+        <f>IF(State!$B$33="quiz","C.   "&amp;INDEX(Steps!$Q$2:$Q$23,State!$B$1),IF(State!$B$33="dials5","Digital and social:  "&amp;TEXT(State!$B$12,"0.0")&amp;" per £1,000",""))</f>
         <v/>
       </c>
       <c r="U15" s="9">
@@ -1766,7 +1765,7 @@
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="T16" s="14">
-        <f>IF(State!$B$33="dial",INDEX(Steps!$V$2:$V$22,State!$B$1),"")</f>
+        <f>IF(State!$B$33="dial",INDEX(Steps!$V$2:$V$23,State!$B$1),"")</f>
         <v/>
       </c>
       <c r="U16" s="15">
@@ -1789,7 +1788,7 @@
     <row r="17" ht="26" customHeight="1"/>
     <row r="18" ht="60" customHeight="1">
       <c r="T18" s="16">
-        <f>IF(State!$B$33="dial",IF(State!$B$37=0,"Tap + to start."&amp;IF(State!$B$15=1," "&amp;INDEX(Steps!$M$2:$M$22,State!$B$1),""),IF(State!$B$41=0,"↑ Higher."&amp;IF(State!$B$15=1," "&amp;INDEX(Steps!$M$2:$M$22,State!$B$1),""),IF(State!$B$41=2,"↓ Lower."&amp;IF(State!$B$15=1," "&amp;INDEX(Steps!$M$2:$M$22,State!$B$1),""),"✓ "&amp;INDEX(Steps!$L$2:$L$22,State!$B$1)))),IF(State!$B$33="quiz",IF(State!$B$39=0,"Pick one.",IF(State!$B$39=State!$B$40,"✓ "&amp;INDEX(Steps!$L$2:$L$22,State!$B$1),"✗ Not quite. "&amp;INDEX(Steps!$M$2:$M$22,State!$B$1))),IF(State!$B$33="dials5",IF(AND(W11="✓",W12="✓",W13="✓",W14="✓",W15="✓"),"✓ "&amp;INDEX(Steps!$L$2:$L$22,State!$B$1),IF(State!$B$15=1,INDEX(Steps!$M$2:$M$22,State!$B$1),"Tap − and + on each channel until five ticks show.")),IF(State!$B$33="tests",IF(State!$B$47=1,"✓ "&amp;INDEX(Steps!$L$2:$L$22,State!$B$1),INDEX(Steps!$M$2:$M$22,State!$B$1)),INDEX(Steps!$L$2:$L$22,State!$B$1)))))</f>
+        <f>IF(State!$B$33="dial",IF(State!$B$37=0,"Tap + to start."&amp;IF(State!$B$15=1," "&amp;INDEX(Steps!$M$2:$M$23,State!$B$1),""),IF(State!$B$41=0,"↑ Higher."&amp;IF(State!$B$15=1," "&amp;INDEX(Steps!$M$2:$M$23,State!$B$1),""),IF(State!$B$41=2,"↓ Lower."&amp;IF(State!$B$15=1," "&amp;INDEX(Steps!$M$2:$M$23,State!$B$1),""),"✓ "&amp;INDEX(Steps!$L$2:$L$23,State!$B$1)))),IF(State!$B$33="quiz",IF(State!$B$39=0,"Pick one.",IF(State!$B$39=State!$B$40,"✓ "&amp;INDEX(Steps!$L$2:$L$23,State!$B$1),"✗ Not quite. "&amp;INDEX(Steps!$M$2:$M$23,State!$B$1))),IF(State!$B$33="dials5",IF(AND(W11="✓",W12="✓",W13="✓",W14="✓",W15="✓"),"✓ "&amp;INDEX(Steps!$L$2:$L$23,State!$B$1),IF(State!$B$15=1,INDEX(Steps!$M$2:$M$23,State!$B$1),"Tap − and + on each channel until five ticks show.")),IF(State!$B$33="tests",IF(State!$B$47=1,"✓ "&amp;INDEX(Steps!$L$2:$L$23,State!$B$1),INDEX(Steps!$M$2:$M$23,State!$B$1)),INDEX(Steps!$L$2:$L$23,State!$B$1)))))</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1798,7 @@
     <row r="22" ht="26" customHeight="1"/>
     <row r="23" ht="24" customHeight="1">
       <c r="T23" s="17">
-        <f>IF(OR(LEFT(T18,1)="✓",State!$B$33="info"),IF(INDEX(Steps!$N$2:$N$22,State!$B$1)="","","Economists call this: "&amp;INDEX(Steps!$N$2:$N$22,State!$B$1)),"")</f>
+        <f>IF(OR(LEFT(T18,1)="✓",State!$B$33="info"),IF(INDEX(Steps!$N$2:$N$23,State!$B$1)="","","Economists call this: "&amp;INDEX(Steps!$N$2:$N$23,State!$B$1)),"")</f>
         <v/>
       </c>
     </row>
@@ -1859,7 +1858,8 @@
       <c r="Y29" s="67" t="n"/>
       <c r="Z29" s="68" t="n"/>
     </row>
-    <row r="31">
+    <row r="30" ht="8" customHeight="1"/>
+    <row r="31" ht="8" customHeight="1">
       <c r="B31" s="6">
         <f>IF(State!$B$33="dial","Tip: −− and ++ move in bigger steps.","")</f>
         <v/>
@@ -1870,22 +1870,866 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="B32" s="1">
+        <f>"Chapter 8  ·  The next pound"</f>
+        <v/>
+      </c>
+      <c r="T32" s="2">
+        <f>REPT("★",State!$B$28)&amp;REPT("☆",10-State!$B$28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="7" customHeight="1">
+      <c r="B33" s="3" t="n"/>
+      <c r="C33" s="3" t="n"/>
+      <c r="D33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="3" t="n"/>
+      <c r="L33" s="3" t="n"/>
+      <c r="M33" s="3" t="n"/>
+      <c r="N33" s="3" t="n"/>
+      <c r="O33" s="3" t="n"/>
+      <c r="P33" s="3" t="n"/>
+      <c r="Q33" s="3" t="n"/>
+      <c r="R33" s="3" t="n"/>
+      <c r="S33" s="3" t="n"/>
+      <c r="T33" s="3" t="n"/>
+      <c r="U33" s="3" t="n"/>
+      <c r="V33" s="3" t="n"/>
+      <c r="W33" s="3" t="n"/>
+      <c r="X33" s="3" t="n"/>
+      <c r="Y33" s="3" t="n"/>
+    </row>
+    <row r="34" ht="40" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Where should the next pound go?</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>The third biscuit never tastes like the first: each extra £1 on a channel earns a little less. Tap − and + to move money. Keep the total. Beat the 2025 plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="8" customHeight="1"/>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="23" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="G37" s="23" t="inlineStr">
+        <is>
+          <t>2025 £k</t>
+        </is>
+      </c>
+      <c r="J37" s="23" t="inlineStr">
+        <is>
+          <t>Your £k</t>
+        </is>
+      </c>
+      <c r="M37" s="23" t="inlineStr"/>
+      <c r="N37" s="23" t="inlineStr"/>
+      <c r="O37" s="23" t="inlineStr">
+        <is>
+          <t>Sign-ups</t>
+        </is>
+      </c>
+      <c r="Q37" s="23" t="inlineStr">
+        <is>
+          <t>Return per £1</t>
+        </is>
+      </c>
+      <c r="T37" s="6" t="inlineStr">
+        <is>
+          <t>Extra sign-ups against the 2025 plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t>DRTV</t>
+        </is>
+      </c>
+      <c r="C38" s="69" t="n"/>
+      <c r="D38" s="69" t="n"/>
+      <c r="E38" s="69" t="n"/>
+      <c r="F38" s="69" t="n"/>
+      <c r="G38" s="25">
+        <f>State!$C$51</f>
+        <v/>
+      </c>
+      <c r="H38" s="69" t="n"/>
+      <c r="I38" s="69" t="n"/>
+      <c r="J38" s="26">
+        <f>IF(State!$B$64=1,State!$E$51,State!$B$51)</f>
+        <v/>
+      </c>
+      <c r="K38" s="69" t="n"/>
+      <c r="L38" s="69" t="n"/>
+      <c r="M38" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N38" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O38" s="28">
+        <f>IF(J38&lt;=0,0,(State!$D$51*State!$C$51*1000/90)/SQRT(State!$C$51)*SQRT(J38))</f>
+        <v/>
+      </c>
+      <c r="P38" s="69" t="n"/>
+      <c r="Q38" s="70">
+        <f>IF(J38&lt;=0,0,O38*State!$B$48/1000/J38)</f>
+        <v/>
+      </c>
+      <c r="R38" s="69" t="n"/>
+      <c r="T38" s="71">
+        <f>O51-SUMPRODUCT(State!$D$51:$D$63,State!$C$51:$C$63)*1000/90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Online video</t>
+        </is>
+      </c>
+      <c r="C39" s="69" t="n"/>
+      <c r="D39" s="69" t="n"/>
+      <c r="E39" s="69" t="n"/>
+      <c r="F39" s="69" t="n"/>
+      <c r="G39" s="25">
+        <f>State!$C$52</f>
+        <v/>
+      </c>
+      <c r="H39" s="69" t="n"/>
+      <c r="I39" s="69" t="n"/>
+      <c r="J39" s="26">
+        <f>IF(State!$B$64=1,State!$E$52,State!$B$52)</f>
+        <v/>
+      </c>
+      <c r="K39" s="69" t="n"/>
+      <c r="L39" s="69" t="n"/>
+      <c r="M39" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N39" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O39" s="28">
+        <f>IF(J39&lt;=0,0,(State!$D$52*State!$C$52*1000/90)/SQRT(State!$C$52)*SQRT(J39))</f>
+        <v/>
+      </c>
+      <c r="P39" s="69" t="n"/>
+      <c r="Q39" s="70">
+        <f>IF(J39&lt;=0,0,O39*State!$B$48/1000/J39)</f>
+        <v/>
+      </c>
+      <c r="R39" s="69" t="n"/>
+      <c r="T39" s="31">
+        <f>IF(ABS(J51-G51)&lt;=10,"Same total as 2025. Good.",IF(J51&gt;G51,"Over budget by £"&amp;TEXT(J51-G51,"#,##0")&amp;"k. Take some back.","Under budget by £"&amp;TEXT(G51-J51,"#,##0")&amp;"k. Spend it."))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t>Radio</t>
+        </is>
+      </c>
+      <c r="C40" s="69" t="n"/>
+      <c r="D40" s="69" t="n"/>
+      <c r="E40" s="69" t="n"/>
+      <c r="F40" s="69" t="n"/>
+      <c r="G40" s="25">
+        <f>State!$C$53</f>
+        <v/>
+      </c>
+      <c r="H40" s="69" t="n"/>
+      <c r="I40" s="69" t="n"/>
+      <c r="J40" s="26">
+        <f>IF(State!$B$64=1,State!$E$53,State!$B$53)</f>
+        <v/>
+      </c>
+      <c r="K40" s="69" t="n"/>
+      <c r="L40" s="69" t="n"/>
+      <c r="M40" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N40" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O40" s="28">
+        <f>IF(J40&lt;=0,0,(State!$D$53*State!$C$53*1000/90)/SQRT(State!$C$53)*SQRT(J40))</f>
+        <v/>
+      </c>
+      <c r="P40" s="69" t="n"/>
+      <c r="Q40" s="70">
+        <f>IF(J40&lt;=0,0,O40*State!$B$48/1000/J40)</f>
+        <v/>
+      </c>
+      <c r="R40" s="69" t="n"/>
+      <c r="T40" s="16">
+        <f>IF(ABS(J51-G51)&gt;10,"Fix the total first.",IF(T38&gt;=1000,"✓ You found "&amp;TEXT(T38,"#,##0")&amp;" extra sign-ups on the same money. The most this table allows is about 2,000.","Move money from the weakest channel to the strongest. Find 1,000 more."))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="24" customHeight="1">
+      <c r="B41" s="24" t="inlineStr">
+        <is>
+          <t>Paid social</t>
+        </is>
+      </c>
+      <c r="C41" s="69" t="n"/>
+      <c r="D41" s="69" t="n"/>
+      <c r="E41" s="69" t="n"/>
+      <c r="F41" s="69" t="n"/>
+      <c r="G41" s="25">
+        <f>State!$C$54</f>
+        <v/>
+      </c>
+      <c r="H41" s="69" t="n"/>
+      <c r="I41" s="69" t="n"/>
+      <c r="J41" s="26">
+        <f>IF(State!$B$64=1,State!$E$54,State!$B$54)</f>
+        <v/>
+      </c>
+      <c r="K41" s="69" t="n"/>
+      <c r="L41" s="69" t="n"/>
+      <c r="M41" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N41" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O41" s="28">
+        <f>IF(J41&lt;=0,0,(State!$D$54*State!$C$54*1000/90)/SQRT(State!$C$54)*SQRT(J41))</f>
+        <v/>
+      </c>
+      <c r="P41" s="69" t="n"/>
+      <c r="Q41" s="70">
+        <f>IF(J41&lt;=0,0,O41*State!$B$48/1000/J41)</f>
+        <v/>
+      </c>
+      <c r="R41" s="69" t="n"/>
+    </row>
+    <row r="42" ht="24" customHeight="1">
+      <c r="B42" s="24" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="C42" s="69" t="n"/>
+      <c r="D42" s="69" t="n"/>
+      <c r="E42" s="69" t="n"/>
+      <c r="F42" s="69" t="n"/>
+      <c r="G42" s="25">
+        <f>State!$C$55</f>
+        <v/>
+      </c>
+      <c r="H42" s="69" t="n"/>
+      <c r="I42" s="69" t="n"/>
+      <c r="J42" s="26">
+        <f>IF(State!$B$64=1,State!$E$55,State!$B$55)</f>
+        <v/>
+      </c>
+      <c r="K42" s="69" t="n"/>
+      <c r="L42" s="69" t="n"/>
+      <c r="M42" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N42" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O42" s="28">
+        <f>IF(J42&lt;=0,0,(State!$D$55*State!$C$55*1000/90)/SQRT(State!$C$55)*SQRT(J42))</f>
+        <v/>
+      </c>
+      <c r="P42" s="69" t="n"/>
+      <c r="Q42" s="70">
+        <f>IF(J42&lt;=0,0,O42*State!$B$48/1000/J42)</f>
+        <v/>
+      </c>
+      <c r="R42" s="69" t="n"/>
+    </row>
+    <row r="43" ht="24" customHeight="1">
+      <c r="B43" s="24" t="inlineStr">
+        <is>
+          <t>Posters</t>
+        </is>
+      </c>
+      <c r="C43" s="69" t="n"/>
+      <c r="D43" s="69" t="n"/>
+      <c r="E43" s="69" t="n"/>
+      <c r="F43" s="69" t="n"/>
+      <c r="G43" s="25">
+        <f>State!$C$56</f>
+        <v/>
+      </c>
+      <c r="H43" s="69" t="n"/>
+      <c r="I43" s="69" t="n"/>
+      <c r="J43" s="26">
+        <f>IF(State!$B$64=1,State!$E$56,State!$B$56)</f>
+        <v/>
+      </c>
+      <c r="K43" s="69" t="n"/>
+      <c r="L43" s="69" t="n"/>
+      <c r="M43" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N43" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O43" s="28">
+        <f>IF(J43&lt;=0,0,(State!$D$56*State!$C$56*1000/90)/SQRT(State!$C$56)*SQRT(J43))</f>
+        <v/>
+      </c>
+      <c r="P43" s="69" t="n"/>
+      <c r="Q43" s="70">
+        <f>IF(J43&lt;=0,0,O43*State!$B$48/1000/J43)</f>
+        <v/>
+      </c>
+      <c r="R43" s="69" t="n"/>
+      <c r="T43" s="32">
+        <f>IF(T38&gt;=1000,"Economists call this: marginal return","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="24" customHeight="1">
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>Digital audio</t>
+        </is>
+      </c>
+      <c r="C44" s="69" t="n"/>
+      <c r="D44" s="69" t="n"/>
+      <c r="E44" s="69" t="n"/>
+      <c r="F44" s="69" t="n"/>
+      <c r="G44" s="25">
+        <f>State!$C$57</f>
+        <v/>
+      </c>
+      <c r="H44" s="69" t="n"/>
+      <c r="I44" s="69" t="n"/>
+      <c r="J44" s="26">
+        <f>IF(State!$B$64=1,State!$E$57,State!$B$57)</f>
+        <v/>
+      </c>
+      <c r="K44" s="69" t="n"/>
+      <c r="L44" s="69" t="n"/>
+      <c r="M44" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N44" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O44" s="28">
+        <f>IF(J44&lt;=0,0,(State!$D$57*State!$C$57*1000/90)/SQRT(State!$C$57)*SQRT(J44))</f>
+        <v/>
+      </c>
+      <c r="P44" s="69" t="n"/>
+      <c r="Q44" s="70">
+        <f>IF(J44&lt;=0,0,O44*State!$B$48/1000/J44)</f>
+        <v/>
+      </c>
+      <c r="R44" s="69" t="n"/>
+    </row>
+    <row r="45" ht="24" customHeight="1">
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="C45" s="69" t="n"/>
+      <c r="D45" s="69" t="n"/>
+      <c r="E45" s="69" t="n"/>
+      <c r="F45" s="69" t="n"/>
+      <c r="G45" s="25">
+        <f>State!$C$58</f>
+        <v/>
+      </c>
+      <c r="H45" s="69" t="n"/>
+      <c r="I45" s="69" t="n"/>
+      <c r="J45" s="26">
+        <f>IF(State!$B$64=1,State!$E$58,State!$B$58)</f>
+        <v/>
+      </c>
+      <c r="K45" s="69" t="n"/>
+      <c r="L45" s="69" t="n"/>
+      <c r="M45" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N45" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O45" s="28">
+        <f>IF(J45&lt;=0,0,(State!$D$58*State!$C$58*1000/90)/SQRT(State!$C$58)*SQRT(J45))</f>
+        <v/>
+      </c>
+      <c r="P45" s="69" t="n"/>
+      <c r="Q45" s="70">
+        <f>IF(J45&lt;=0,0,O45*State!$B$48/1000/J45)</f>
+        <v/>
+      </c>
+      <c r="R45" s="69" t="n"/>
+      <c r="T45" s="33" t="inlineStr">
+        <is>
+          <t>The average £1 returned £1.66. The last £1 returned 82p. Should we add £1m to the same plan?</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="24" customHeight="1">
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>Paid search</t>
+        </is>
+      </c>
+      <c r="C46" s="69" t="n"/>
+      <c r="D46" s="69" t="n"/>
+      <c r="E46" s="69" t="n"/>
+      <c r="F46" s="69" t="n"/>
+      <c r="G46" s="25">
+        <f>State!$C$59</f>
+        <v/>
+      </c>
+      <c r="H46" s="69" t="n"/>
+      <c r="I46" s="69" t="n"/>
+      <c r="J46" s="26">
+        <f>IF(State!$B$64=1,State!$E$59,State!$B$59)</f>
+        <v/>
+      </c>
+      <c r="K46" s="69" t="n"/>
+      <c r="L46" s="69" t="n"/>
+      <c r="M46" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N46" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O46" s="28">
+        <f>IF(J46&lt;=0,0,(State!$D$59*State!$C$59*1000/90)/SQRT(State!$C$59)*SQRT(J46))</f>
+        <v/>
+      </c>
+      <c r="P46" s="69" t="n"/>
+      <c r="Q46" s="70">
+        <f>IF(J46&lt;=0,0,O46*State!$B$48/1000/J46)</f>
+        <v/>
+      </c>
+      <c r="R46" s="69" t="n"/>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C47" s="69" t="n"/>
+      <c r="D47" s="69" t="n"/>
+      <c r="E47" s="69" t="n"/>
+      <c r="F47" s="69" t="n"/>
+      <c r="G47" s="25">
+        <f>State!$C$60</f>
+        <v/>
+      </c>
+      <c r="H47" s="69" t="n"/>
+      <c r="I47" s="69" t="n"/>
+      <c r="J47" s="26">
+        <f>IF(State!$B$64=1,State!$E$60,State!$B$60)</f>
+        <v/>
+      </c>
+      <c r="K47" s="69" t="n"/>
+      <c r="L47" s="69" t="n"/>
+      <c r="M47" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N47" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O47" s="28">
+        <f>IF(J47&lt;=0,0,(State!$D$60*State!$C$60*1000/90)/SQRT(State!$C$60)*SQRT(J47))</f>
+        <v/>
+      </c>
+      <c r="P47" s="69" t="n"/>
+      <c r="Q47" s="70">
+        <f>IF(J47&lt;=0,0,O47*State!$B$48/1000/J47)</f>
+        <v/>
+      </c>
+      <c r="R47" s="69" t="n"/>
+      <c r="T47" s="34" t="inlineStr">
+        <is>
+          <t>A.   Not yet: move money first</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24" customHeight="1">
+      <c r="B48" s="24" t="inlineStr">
+        <is>
+          <t>Telemarketing</t>
+        </is>
+      </c>
+      <c r="C48" s="69" t="n"/>
+      <c r="D48" s="69" t="n"/>
+      <c r="E48" s="69" t="n"/>
+      <c r="F48" s="69" t="n"/>
+      <c r="G48" s="25">
+        <f>State!$C$61</f>
+        <v/>
+      </c>
+      <c r="H48" s="69" t="n"/>
+      <c r="I48" s="69" t="n"/>
+      <c r="J48" s="26">
+        <f>IF(State!$B$64=1,State!$E$61,State!$B$61)</f>
+        <v/>
+      </c>
+      <c r="K48" s="69" t="n"/>
+      <c r="L48" s="69" t="n"/>
+      <c r="M48" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N48" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O48" s="28">
+        <f>IF(J48&lt;=0,0,(State!$D$61*State!$C$61*1000/90)/SQRT(State!$C$61)*SQRT(J48))</f>
+        <v/>
+      </c>
+      <c r="P48" s="69" t="n"/>
+      <c r="Q48" s="70">
+        <f>IF(J48&lt;=0,0,O48*State!$B$48/1000/J48)</f>
+        <v/>
+      </c>
+      <c r="R48" s="69" t="n"/>
+      <c r="T48" s="34" t="inlineStr">
+        <is>
+          <t>B.   Yes, every £1 returns £1.66</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="24" customHeight="1">
+      <c r="B49" s="24" t="inlineStr">
+        <is>
+          <t>Direct mail</t>
+        </is>
+      </c>
+      <c r="C49" s="69" t="n"/>
+      <c r="D49" s="69" t="n"/>
+      <c r="E49" s="69" t="n"/>
+      <c r="F49" s="69" t="n"/>
+      <c r="G49" s="25">
+        <f>State!$C$62</f>
+        <v/>
+      </c>
+      <c r="H49" s="69" t="n"/>
+      <c r="I49" s="69" t="n"/>
+      <c r="J49" s="26">
+        <f>IF(State!$B$64=1,State!$E$62,State!$B$62)</f>
+        <v/>
+      </c>
+      <c r="K49" s="69" t="n"/>
+      <c r="L49" s="69" t="n"/>
+      <c r="M49" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N49" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O49" s="28">
+        <f>IF(J49&lt;=0,0,(State!$D$62*State!$C$62*1000/90)/SQRT(State!$C$62)*SQRT(J49))</f>
+        <v/>
+      </c>
+      <c r="P49" s="69" t="n"/>
+      <c r="Q49" s="70">
+        <f>IF(J49&lt;=0,0,O49*State!$B$48/1000/J49)</f>
+        <v/>
+      </c>
+      <c r="R49" s="69" t="n"/>
+      <c r="T49" s="34" t="inlineStr">
+        <is>
+          <t>C.   No, cut everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24" customHeight="1">
+      <c r="B50" s="24" t="inlineStr">
+        <is>
+          <t>Door drops</t>
+        </is>
+      </c>
+      <c r="C50" s="69" t="n"/>
+      <c r="D50" s="69" t="n"/>
+      <c r="E50" s="69" t="n"/>
+      <c r="F50" s="69" t="n"/>
+      <c r="G50" s="25">
+        <f>State!$C$63</f>
+        <v/>
+      </c>
+      <c r="H50" s="69" t="n"/>
+      <c r="I50" s="69" t="n"/>
+      <c r="J50" s="26">
+        <f>IF(State!$B$64=1,State!$E$63,State!$B$63)</f>
+        <v/>
+      </c>
+      <c r="K50" s="69" t="n"/>
+      <c r="L50" s="69" t="n"/>
+      <c r="M50" s="27" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="N50" s="27" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="O50" s="28">
+        <f>IF(J50&lt;=0,0,(State!$D$63*State!$C$63*1000/90)/SQRT(State!$C$63)*SQRT(J50))</f>
+        <v/>
+      </c>
+      <c r="P50" s="69" t="n"/>
+      <c r="Q50" s="70">
+        <f>IF(J50&lt;=0,0,O50*State!$B$48/1000/J50)</f>
+        <v/>
+      </c>
+      <c r="R50" s="69" t="n"/>
+      <c r="T50" s="16">
+        <f>IF(State!$B$24=0,"Pick one.",IF(State!$B$24=State!$C$24,"✓ Moving money between channels was worth about £1.1m before adding a single pound.","✗ Not quite. The average pound looks great. The next pound does not."))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="B51" s="35" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="G51" s="36">
+        <f>SUM(G38:G50)</f>
+        <v/>
+      </c>
+      <c r="J51" s="37">
+        <f>SUM(J38:J50)</f>
+        <v/>
+      </c>
+      <c r="O51" s="36">
+        <f>SUM(O38:O50)</f>
+        <v/>
+      </c>
+      <c r="Q51" s="72">
+        <f>O51*State!$B$48/1000/J51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>Each channel's curve is set so the 2025 plan gives exactly Wave 1's return. Double a channel's spend and you get 41% more sign-ups, not double. AP's real curves differ by channel, so their plan gained 12,300 sign-ups with them and about 600 here. The direction is the lesson.</t>
+        </is>
+      </c>
+      <c r="T52" s="32">
+        <f>IF(LEFT(T50,1)="✓","Economists call this: Marginal return","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1"/>
+    <row r="55" ht="34" customHeight="1">
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t>◀  Back</t>
+        </is>
+      </c>
+      <c r="C55" s="67" t="n"/>
+      <c r="D55" s="67" t="n"/>
+      <c r="E55" s="68" t="n"/>
+      <c r="G55" s="19">
+        <f>IF(State!$B$64=1,"Back to my plan","Show AP's plan")</f>
+        <v/>
+      </c>
+      <c r="H55" s="67" t="n"/>
+      <c r="I55" s="67" t="n"/>
+      <c r="J55" s="68" t="n"/>
+      <c r="L55" s="19" t="inlineStr">
+        <is>
+          <t>Reset plan</t>
+        </is>
+      </c>
+      <c r="M55" s="67" t="n"/>
+      <c r="N55" s="67" t="n"/>
+      <c r="O55" s="68" t="n"/>
+      <c r="T55" s="21" t="inlineStr">
+        <is>
+          <t>Next  ▶</t>
+        </is>
+      </c>
+      <c r="U55" s="67" t="n"/>
+      <c r="V55" s="67" t="n"/>
+      <c r="W55" s="67" t="n"/>
+      <c r="X55" s="67" t="n"/>
+      <c r="Y55" s="67" t="n"/>
+      <c r="Z55" s="68" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="104">
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="G55:J55"/>
+    <mergeCell ref="T27:Z27"/>
+    <mergeCell ref="B42:F42"/>
+    <mergeCell ref="Q51:R51"/>
+    <mergeCell ref="B35:Z35"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="J50:L50"/>
+    <mergeCell ref="N37"/>
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="J46:L46"/>
+    <mergeCell ref="G50:I50"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="J39:L39"/>
+    <mergeCell ref="J48:L48"/>
+    <mergeCell ref="Q49:R49"/>
+    <mergeCell ref="T25:Z25"/>
+    <mergeCell ref="T55:Z55"/>
+    <mergeCell ref="J38:L38"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="L55:O55"/>
+    <mergeCell ref="T2:Z2"/>
+    <mergeCell ref="J40:L40"/>
+    <mergeCell ref="M37"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="Q37:R37"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="O45:P45"/>
+    <mergeCell ref="T50:Z51"/>
+    <mergeCell ref="Q39:R39"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="Q29:R29"/>
+    <mergeCell ref="Q38:R38"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="J43:L43"/>
+    <mergeCell ref="T29:Z29"/>
+    <mergeCell ref="G51:I51"/>
+    <mergeCell ref="Q31:R31"/>
     <mergeCell ref="B7:Z7"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="T23:Z23"/>
-    <mergeCell ref="T27:Z27"/>
-    <mergeCell ref="Q29:R29"/>
-    <mergeCell ref="B5:Z5"/>
+    <mergeCell ref="Q40:R40"/>
+    <mergeCell ref="G41:I41"/>
+    <mergeCell ref="J42:L42"/>
+    <mergeCell ref="O51:P51"/>
+    <mergeCell ref="G43:I43"/>
+    <mergeCell ref="J44:L44"/>
+    <mergeCell ref="T40:Z42"/>
+    <mergeCell ref="J37:L37"/>
     <mergeCell ref="B31:M31"/>
     <mergeCell ref="B29:E29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="T2:Z2"/>
+    <mergeCell ref="B45:F45"/>
     <mergeCell ref="L29:O29"/>
-    <mergeCell ref="T25:Z25"/>
-    <mergeCell ref="T29:Z29"/>
-    <mergeCell ref="Q31:R31"/>
+    <mergeCell ref="B34:Z34"/>
+    <mergeCell ref="B47:F47"/>
+    <mergeCell ref="Q42:R42"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B48:F48"/>
+    <mergeCell ref="G45:I45"/>
+    <mergeCell ref="J47:L47"/>
+    <mergeCell ref="T32:Z32"/>
+    <mergeCell ref="G47:I47"/>
+    <mergeCell ref="G44:I44"/>
+    <mergeCell ref="G46:I46"/>
+    <mergeCell ref="O46:P46"/>
+    <mergeCell ref="G40:I40"/>
+    <mergeCell ref="Q46:R46"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="Q48:R48"/>
+    <mergeCell ref="Q45:R45"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="Q41:R41"/>
+    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="Q47:R47"/>
+    <mergeCell ref="T23:Z23"/>
+    <mergeCell ref="T45:Z46"/>
+    <mergeCell ref="J49:L49"/>
+    <mergeCell ref="Q43:R43"/>
+    <mergeCell ref="J45:L45"/>
+    <mergeCell ref="G49:I49"/>
+    <mergeCell ref="O49:P49"/>
+    <mergeCell ref="B5:Z5"/>
+    <mergeCell ref="Q50:R50"/>
+    <mergeCell ref="J51:L51"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="O50:P50"/>
+    <mergeCell ref="Q44:R44"/>
+    <mergeCell ref="B32:M32"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B52:R53"/>
+    <mergeCell ref="B51:F51"/>
+    <mergeCell ref="G39:I39"/>
+    <mergeCell ref="G48:I48"/>
+    <mergeCell ref="O37:P37"/>
+    <mergeCell ref="B41:F41"/>
     <mergeCell ref="T18:Z21"/>
   </mergeCells>
   <conditionalFormatting sqref="B3:Y3">
@@ -1971,6 +2815,59 @@
       <formula>State!$B$33="info"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B33:Y33">
+    <cfRule type="expression" priority="20" dxfId="0">
+      <formula>COLUMN()-1&lt;=State!$B$31</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J38:J50">
+    <cfRule type="dataBar" priority="21">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="1600"/>
+        <color rgb="00009CEE"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T39">
+    <cfRule type="expression" priority="22" dxfId="9">
+      <formula>ISNUMBER(SEARCH("Good",T39))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="10">
+      <formula>NOT(ISNUMBER(SEARCH("Good",T39)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T40">
+    <cfRule type="expression" priority="24" dxfId="6">
+      <formula>LEFT(T40,1)="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="25" dxfId="7">
+      <formula>LEFT(T40,1)&lt;&gt;"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T47">
+    <cfRule type="expression" priority="26" dxfId="4">
+      <formula>State!$B$24=1</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T48">
+    <cfRule type="expression" priority="27" dxfId="4">
+      <formula>State!$B$24=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T49">
+    <cfRule type="expression" priority="28" dxfId="4">
+      <formula>State!$B$24=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T50">
+    <cfRule type="expression" priority="29" dxfId="6">
+      <formula>LEFT(T50,1)="✓"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="7">
+      <formula>LEFT(T50,1)="✗"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>
@@ -1991,167 +2888,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="2">
-      <c r="B2" s="50" t="inlineStr">
-        <is>
-          <t>Room notes: running the game with a team in 45 minutes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="65" t="inlineStr">
-        <is>
-          <t>For the person leading. Unhide from the sheet list. The answers are here, so do not share the screen with this tab open.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="B5" s="66" t="inlineStr">
-        <is>
-          <t>0 to 5</t>
-        </is>
-      </c>
-      <c r="C5" s="41" t="inlineStr">
-        <is>
-          <t>Open Play on the big screen. Chapter 1, one person tapping. Ask the room what made the spikes before anyone taps.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="B6" s="66" t="inlineStr">
-        <is>
-          <t>5 to 15</t>
-        </is>
-      </c>
-      <c r="C6" s="41" t="inlineStr">
-        <is>
-          <t>Chapters 2 and 3 together. Ask for a show of hands before each number: higher or lower than a thousand? The base surprises people. Let it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="B7" s="66" t="inlineStr">
-        <is>
-          <t>15 to 25</t>
-        </is>
-      </c>
-      <c r="C7" s="41" t="inlineStr">
-        <is>
-          <t>Chapter 4. Ask the room to guess the memory before you touch it. Most say 20%. Show what 80% does. Name adstock only after the line fits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="B8" s="66" t="inlineStr">
-        <is>
-          <t>25 to 32</t>
-        </is>
-      </c>
-      <c r="C8" s="41" t="inlineStr">
-        <is>
-          <t>Chapter 5. Add the halo, then read the 42% step out loud and stop. Let the room say what it means for next year.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="B9" s="66" t="inlineStr">
-        <is>
-          <t>32 to 38</t>
-        </is>
-      </c>
-      <c r="C9" s="41" t="inlineStr">
-        <is>
-          <t>Chapter 6 in pairs on laptops. The point is the catch, not the numbers. Ask: which channel are you least sure of, and why?</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="B10" s="66" t="inlineStr">
-        <is>
-          <t>38 to 45</t>
-        </is>
-      </c>
-      <c r="C10" s="41" t="inlineStr">
-        <is>
-          <t>Chapter 8 as a race: first to 1,000 extra sign-ups on the same money. Close on average versus last pound. Chapters 9 and 10 are homework.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="49" customHeight="1">
-      <c r="B11" s="66" t="inlineStr">
-        <is>
-          <t>Answer key</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="inlineStr">
-        <is>
-          <t>Base 876. Brake 952. Sale 7,598. Adverts 16.1 per £1,000, memory 80%. Halo 2.86 per £1,000. Channels: TV 17.0, Online video 17.4, Radio 17.4, Posters 6.1, Digital and social 17.6. Every quiz answer is A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="49" customHeight="1">
-      <c r="B12" s="66" t="inlineStr">
-        <is>
-          <t>If asked "is this just correlation?"</t>
-        </is>
-      </c>
-      <c r="C12" s="41" t="inlineStr">
-        <is>
-          <t>Partly, and AP say so. Three things make it more: it controls for everything at once, it is tested on weeks it never saw, and channels that stopped (Race for Life TV after 2024) let it see what happens without them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="B13" s="66" t="inlineStr">
-        <is>
-          <t>If asked "the halo felt too big"</t>
-        </is>
-      </c>
-      <c r="C13" s="41" t="inlineStr">
-        <is>
-          <t>It did, and AP rebuilt it. They now measure Committed Giving as one block. The halo fell and is still 5% of 2025 sign-ups and 9,139 of the 2025 decline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="B14" s="66" t="inlineStr">
-        <is>
-          <t>Budget chapter</t>
-        </is>
-      </c>
-      <c r="C14" s="41" t="inlineStr">
-        <is>
-          <t>Best possible on the game's curves is about 2,000 extra: cut posters and telemarketing, add DRTV and online video. AP's own plan shows the same direction.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9"/>
-  <headerFooter>
-    <oddHeader>&amp;LCRUK CONFIDENTIAL, INTERNAL USE ONLY</oddHeader>
-    <oddFooter>&amp;LThe Econometrics Game v3&amp;RAndrew Rajanathan, CRUK M&amp;&amp;D</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet11">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2363,963 +3099,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet2">
-    <tabColor rgb="00E60078"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="B2:Z29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="5.2" customWidth="1" min="2" max="2"/>
-    <col width="5.2" customWidth="1" min="3" max="3"/>
-    <col width="5.2" customWidth="1" min="4" max="4"/>
-    <col width="5.2" customWidth="1" min="5" max="5"/>
-    <col width="5.2" customWidth="1" min="6" max="6"/>
-    <col width="5.2" customWidth="1" min="7" max="7"/>
-    <col width="5.2" customWidth="1" min="8" max="8"/>
-    <col width="5.2" customWidth="1" min="9" max="9"/>
-    <col width="5.2" customWidth="1" min="10" max="10"/>
-    <col width="5.2" customWidth="1" min="11" max="11"/>
-    <col width="5.2" customWidth="1" min="12" max="12"/>
-    <col width="5.2" customWidth="1" min="13" max="13"/>
-    <col width="5.2" customWidth="1" min="14" max="14"/>
-    <col width="5.2" customWidth="1" min="15" max="15"/>
-    <col width="5.2" customWidth="1" min="16" max="16"/>
-    <col width="5.2" customWidth="1" min="17" max="17"/>
-    <col width="5.2" customWidth="1" min="18" max="18"/>
-    <col width="2" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
-    <col width="5.5" customWidth="1" min="21" max="21"/>
-    <col width="5.5" customWidth="1" min="22" max="22"/>
-    <col width="5.5" customWidth="1" min="23" max="23"/>
-    <col width="7" customWidth="1" min="24" max="24"/>
-    <col width="7" customWidth="1" min="25" max="25"/>
-    <col width="7" customWidth="1" min="26" max="26"/>
-    <col width="2" customWidth="1" min="27" max="27"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="8" customHeight="1"/>
-    <row r="2" ht="20" customHeight="1">
-      <c r="B2" s="1">
-        <f>"Chapter 8  ·  The next pound"</f>
-        <v/>
-      </c>
-      <c r="T2" s="2">
-        <f>REPT("★",State!$B$28)&amp;REPT("☆",10-State!$B$28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3" ht="7" customHeight="1">
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
-      <c r="O3" s="3" t="n"/>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
-      <c r="R3" s="3" t="n"/>
-      <c r="S3" s="3" t="n"/>
-      <c r="T3" s="3" t="n"/>
-      <c r="U3" s="3" t="n"/>
-      <c r="V3" s="3" t="n"/>
-      <c r="W3" s="3" t="n"/>
-      <c r="X3" s="3" t="n"/>
-      <c r="Y3" s="3" t="n"/>
-    </row>
-    <row r="4" ht="8" customHeight="1"/>
-    <row r="5" ht="40" customHeight="1">
-      <c r="B5" s="4">
-        <f>"Where should the next pound go?"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="6" customHeight="1"/>
-    <row r="7" ht="48" customHeight="1">
-      <c r="B7" s="5">
-        <f>"The third biscuit never tastes like the first: each extra £1 on a channel earns a little less. Tap − and + to move money. Keep the total. Beat the 2025 plan."</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="8" customHeight="1"/>
-    <row r="9" ht="10" customHeight="1"/>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="23" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="G10" s="23" t="inlineStr">
-        <is>
-          <t>2025 £k</t>
-        </is>
-      </c>
-      <c r="J10" s="23" t="inlineStr">
-        <is>
-          <t>Your £k</t>
-        </is>
-      </c>
-      <c r="M10" s="23" t="inlineStr"/>
-      <c r="N10" s="23" t="inlineStr"/>
-      <c r="O10" s="23" t="inlineStr">
-        <is>
-          <t>Sign-ups</t>
-        </is>
-      </c>
-      <c r="Q10" s="23" t="inlineStr">
-        <is>
-          <t>Return per £1</t>
-        </is>
-      </c>
-      <c r="T10" s="6" t="inlineStr">
-        <is>
-          <t>Extra sign-ups against the 2025 plan</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>DRTV</t>
-        </is>
-      </c>
-      <c r="C11" s="69" t="n"/>
-      <c r="D11" s="69" t="n"/>
-      <c r="E11" s="69" t="n"/>
-      <c r="F11" s="69" t="n"/>
-      <c r="G11" s="25">
-        <f>State!$C$51</f>
-        <v/>
-      </c>
-      <c r="H11" s="69" t="n"/>
-      <c r="I11" s="69" t="n"/>
-      <c r="J11" s="26">
-        <f>IF(State!$B$64=1,State!$E$51,State!$B$51)</f>
-        <v/>
-      </c>
-      <c r="K11" s="69" t="n"/>
-      <c r="L11" s="69" t="n"/>
-      <c r="M11" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N11" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O11" s="28">
-        <f>IF(J11&lt;=0,0,(State!$D$51*State!$C$51*1000/90)/SQRT(State!$C$51)*SQRT(J11))</f>
-        <v/>
-      </c>
-      <c r="P11" s="69" t="n"/>
-      <c r="Q11" s="70">
-        <f>IF(J11&lt;=0,0,O11*State!$B$48/1000/J11)</f>
-        <v/>
-      </c>
-      <c r="R11" s="69" t="n"/>
-      <c r="T11" s="71">
-        <f>O24-SUMPRODUCT(State!$D$51:$D$63,State!$C$51:$C$63)*1000/90</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="24" t="inlineStr">
-        <is>
-          <t>Online video</t>
-        </is>
-      </c>
-      <c r="C12" s="69" t="n"/>
-      <c r="D12" s="69" t="n"/>
-      <c r="E12" s="69" t="n"/>
-      <c r="F12" s="69" t="n"/>
-      <c r="G12" s="25">
-        <f>State!$C$52</f>
-        <v/>
-      </c>
-      <c r="H12" s="69" t="n"/>
-      <c r="I12" s="69" t="n"/>
-      <c r="J12" s="26">
-        <f>IF(State!$B$64=1,State!$E$52,State!$B$52)</f>
-        <v/>
-      </c>
-      <c r="K12" s="69" t="n"/>
-      <c r="L12" s="69" t="n"/>
-      <c r="M12" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N12" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O12" s="28">
-        <f>IF(J12&lt;=0,0,(State!$D$52*State!$C$52*1000/90)/SQRT(State!$C$52)*SQRT(J12))</f>
-        <v/>
-      </c>
-      <c r="P12" s="69" t="n"/>
-      <c r="Q12" s="70">
-        <f>IF(J12&lt;=0,0,O12*State!$B$48/1000/J12)</f>
-        <v/>
-      </c>
-      <c r="R12" s="69" t="n"/>
-      <c r="T12" s="31">
-        <f>IF(ABS(J24-G24)&lt;=10,"Same total as 2025. Good.",IF(J24&gt;G24,"Over budget by £"&amp;TEXT(J24-G24,"#,##0")&amp;"k. Take some back.","Under budget by £"&amp;TEXT(G24-J24,"#,##0")&amp;"k. Spend it."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="C13" s="69" t="n"/>
-      <c r="D13" s="69" t="n"/>
-      <c r="E13" s="69" t="n"/>
-      <c r="F13" s="69" t="n"/>
-      <c r="G13" s="25">
-        <f>State!$C$53</f>
-        <v/>
-      </c>
-      <c r="H13" s="69" t="n"/>
-      <c r="I13" s="69" t="n"/>
-      <c r="J13" s="26">
-        <f>IF(State!$B$64=1,State!$E$53,State!$B$53)</f>
-        <v/>
-      </c>
-      <c r="K13" s="69" t="n"/>
-      <c r="L13" s="69" t="n"/>
-      <c r="M13" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N13" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O13" s="28">
-        <f>IF(J13&lt;=0,0,(State!$D$53*State!$C$53*1000/90)/SQRT(State!$C$53)*SQRT(J13))</f>
-        <v/>
-      </c>
-      <c r="P13" s="69" t="n"/>
-      <c r="Q13" s="70">
-        <f>IF(J13&lt;=0,0,O13*State!$B$48/1000/J13)</f>
-        <v/>
-      </c>
-      <c r="R13" s="69" t="n"/>
-      <c r="T13" s="16">
-        <f>IF(ABS(J24-G24)&gt;10,"Fix the total first.",IF(T11&gt;=1000,"✓ You found "&amp;TEXT(T11,"#,##0")&amp;" extra sign-ups on the same money. The most this table allows is about 2,000.","Move money from the weakest channel to the strongest. Find 1,000 more."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="B14" s="24" t="inlineStr">
-        <is>
-          <t>Paid social</t>
-        </is>
-      </c>
-      <c r="C14" s="69" t="n"/>
-      <c r="D14" s="69" t="n"/>
-      <c r="E14" s="69" t="n"/>
-      <c r="F14" s="69" t="n"/>
-      <c r="G14" s="25">
-        <f>State!$C$54</f>
-        <v/>
-      </c>
-      <c r="H14" s="69" t="n"/>
-      <c r="I14" s="69" t="n"/>
-      <c r="J14" s="26">
-        <f>IF(State!$B$64=1,State!$E$54,State!$B$54)</f>
-        <v/>
-      </c>
-      <c r="K14" s="69" t="n"/>
-      <c r="L14" s="69" t="n"/>
-      <c r="M14" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N14" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O14" s="28">
-        <f>IF(J14&lt;=0,0,(State!$D$54*State!$C$54*1000/90)/SQRT(State!$C$54)*SQRT(J14))</f>
-        <v/>
-      </c>
-      <c r="P14" s="69" t="n"/>
-      <c r="Q14" s="70">
-        <f>IF(J14&lt;=0,0,O14*State!$B$48/1000/J14)</f>
-        <v/>
-      </c>
-      <c r="R14" s="69" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="B15" s="24" t="inlineStr">
-        <is>
-          <t>Regional</t>
-        </is>
-      </c>
-      <c r="C15" s="69" t="n"/>
-      <c r="D15" s="69" t="n"/>
-      <c r="E15" s="69" t="n"/>
-      <c r="F15" s="69" t="n"/>
-      <c r="G15" s="25">
-        <f>State!$C$55</f>
-        <v/>
-      </c>
-      <c r="H15" s="69" t="n"/>
-      <c r="I15" s="69" t="n"/>
-      <c r="J15" s="26">
-        <f>IF(State!$B$64=1,State!$E$55,State!$B$55)</f>
-        <v/>
-      </c>
-      <c r="K15" s="69" t="n"/>
-      <c r="L15" s="69" t="n"/>
-      <c r="M15" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N15" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O15" s="28">
-        <f>IF(J15&lt;=0,0,(State!$D$55*State!$C$55*1000/90)/SQRT(State!$C$55)*SQRT(J15))</f>
-        <v/>
-      </c>
-      <c r="P15" s="69" t="n"/>
-      <c r="Q15" s="70">
-        <f>IF(J15&lt;=0,0,O15*State!$B$48/1000/J15)</f>
-        <v/>
-      </c>
-      <c r="R15" s="69" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="B16" s="24" t="inlineStr">
-        <is>
-          <t>Posters</t>
-        </is>
-      </c>
-      <c r="C16" s="69" t="n"/>
-      <c r="D16" s="69" t="n"/>
-      <c r="E16" s="69" t="n"/>
-      <c r="F16" s="69" t="n"/>
-      <c r="G16" s="25">
-        <f>State!$C$56</f>
-        <v/>
-      </c>
-      <c r="H16" s="69" t="n"/>
-      <c r="I16" s="69" t="n"/>
-      <c r="J16" s="26">
-        <f>IF(State!$B$64=1,State!$E$56,State!$B$56)</f>
-        <v/>
-      </c>
-      <c r="K16" s="69" t="n"/>
-      <c r="L16" s="69" t="n"/>
-      <c r="M16" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N16" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O16" s="28">
-        <f>IF(J16&lt;=0,0,(State!$D$56*State!$C$56*1000/90)/SQRT(State!$C$56)*SQRT(J16))</f>
-        <v/>
-      </c>
-      <c r="P16" s="69" t="n"/>
-      <c r="Q16" s="70">
-        <f>IF(J16&lt;=0,0,O16*State!$B$48/1000/J16)</f>
-        <v/>
-      </c>
-      <c r="R16" s="69" t="n"/>
-      <c r="T16" s="32">
-        <f>IF(T11&gt;=1000,"Economists call this: marginal return","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="B17" s="24" t="inlineStr">
-        <is>
-          <t>Digital audio</t>
-        </is>
-      </c>
-      <c r="C17" s="69" t="n"/>
-      <c r="D17" s="69" t="n"/>
-      <c r="E17" s="69" t="n"/>
-      <c r="F17" s="69" t="n"/>
-      <c r="G17" s="25">
-        <f>State!$C$57</f>
-        <v/>
-      </c>
-      <c r="H17" s="69" t="n"/>
-      <c r="I17" s="69" t="n"/>
-      <c r="J17" s="26">
-        <f>IF(State!$B$64=1,State!$E$57,State!$B$57)</f>
-        <v/>
-      </c>
-      <c r="K17" s="69" t="n"/>
-      <c r="L17" s="69" t="n"/>
-      <c r="M17" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N17" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O17" s="28">
-        <f>IF(J17&lt;=0,0,(State!$D$57*State!$C$57*1000/90)/SQRT(State!$C$57)*SQRT(J17))</f>
-        <v/>
-      </c>
-      <c r="P17" s="69" t="n"/>
-      <c r="Q17" s="70">
-        <f>IF(J17&lt;=0,0,O17*State!$B$48/1000/J17)</f>
-        <v/>
-      </c>
-      <c r="R17" s="69" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>Display</t>
-        </is>
-      </c>
-      <c r="C18" s="69" t="n"/>
-      <c r="D18" s="69" t="n"/>
-      <c r="E18" s="69" t="n"/>
-      <c r="F18" s="69" t="n"/>
-      <c r="G18" s="25">
-        <f>State!$C$58</f>
-        <v/>
-      </c>
-      <c r="H18" s="69" t="n"/>
-      <c r="I18" s="69" t="n"/>
-      <c r="J18" s="26">
-        <f>IF(State!$B$64=1,State!$E$58,State!$B$58)</f>
-        <v/>
-      </c>
-      <c r="K18" s="69" t="n"/>
-      <c r="L18" s="69" t="n"/>
-      <c r="M18" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N18" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O18" s="28">
-        <f>IF(J18&lt;=0,0,(State!$D$58*State!$C$58*1000/90)/SQRT(State!$C$58)*SQRT(J18))</f>
-        <v/>
-      </c>
-      <c r="P18" s="69" t="n"/>
-      <c r="Q18" s="70">
-        <f>IF(J18&lt;=0,0,O18*State!$B$48/1000/J18)</f>
-        <v/>
-      </c>
-      <c r="R18" s="69" t="n"/>
-      <c r="T18" s="33" t="inlineStr">
-        <is>
-          <t>The average £1 returned £1.66. The last £1 returned 82p. Should we add £1m to the same plan?</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="B19" s="24" t="inlineStr">
-        <is>
-          <t>Paid search</t>
-        </is>
-      </c>
-      <c r="C19" s="69" t="n"/>
-      <c r="D19" s="69" t="n"/>
-      <c r="E19" s="69" t="n"/>
-      <c r="F19" s="69" t="n"/>
-      <c r="G19" s="25">
-        <f>State!$C$59</f>
-        <v/>
-      </c>
-      <c r="H19" s="69" t="n"/>
-      <c r="I19" s="69" t="n"/>
-      <c r="J19" s="26">
-        <f>IF(State!$B$64=1,State!$E$59,State!$B$59)</f>
-        <v/>
-      </c>
-      <c r="K19" s="69" t="n"/>
-      <c r="L19" s="69" t="n"/>
-      <c r="M19" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N19" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O19" s="28">
-        <f>IF(J19&lt;=0,0,(State!$D$59*State!$C$59*1000/90)/SQRT(State!$C$59)*SQRT(J19))</f>
-        <v/>
-      </c>
-      <c r="P19" s="69" t="n"/>
-      <c r="Q19" s="70">
-        <f>IF(J19&lt;=0,0,O19*State!$B$48/1000/J19)</f>
-        <v/>
-      </c>
-      <c r="R19" s="69" t="n"/>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="B20" s="24" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="C20" s="69" t="n"/>
-      <c r="D20" s="69" t="n"/>
-      <c r="E20" s="69" t="n"/>
-      <c r="F20" s="69" t="n"/>
-      <c r="G20" s="25">
-        <f>State!$C$60</f>
-        <v/>
-      </c>
-      <c r="H20" s="69" t="n"/>
-      <c r="I20" s="69" t="n"/>
-      <c r="J20" s="26">
-        <f>IF(State!$B$64=1,State!$E$60,State!$B$60)</f>
-        <v/>
-      </c>
-      <c r="K20" s="69" t="n"/>
-      <c r="L20" s="69" t="n"/>
-      <c r="M20" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N20" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O20" s="28">
-        <f>IF(J20&lt;=0,0,(State!$D$60*State!$C$60*1000/90)/SQRT(State!$C$60)*SQRT(J20))</f>
-        <v/>
-      </c>
-      <c r="P20" s="69" t="n"/>
-      <c r="Q20" s="70">
-        <f>IF(J20&lt;=0,0,O20*State!$B$48/1000/J20)</f>
-        <v/>
-      </c>
-      <c r="R20" s="69" t="n"/>
-      <c r="T20" s="34" t="inlineStr">
-        <is>
-          <t>A.   Not yet: move money first</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="B21" s="24" t="inlineStr">
-        <is>
-          <t>Telemarketing</t>
-        </is>
-      </c>
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="69" t="n"/>
-      <c r="E21" s="69" t="n"/>
-      <c r="F21" s="69" t="n"/>
-      <c r="G21" s="25">
-        <f>State!$C$61</f>
-        <v/>
-      </c>
-      <c r="H21" s="69" t="n"/>
-      <c r="I21" s="69" t="n"/>
-      <c r="J21" s="26">
-        <f>IF(State!$B$64=1,State!$E$61,State!$B$61)</f>
-        <v/>
-      </c>
-      <c r="K21" s="69" t="n"/>
-      <c r="L21" s="69" t="n"/>
-      <c r="M21" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N21" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O21" s="28">
-        <f>IF(J21&lt;=0,0,(State!$D$61*State!$C$61*1000/90)/SQRT(State!$C$61)*SQRT(J21))</f>
-        <v/>
-      </c>
-      <c r="P21" s="69" t="n"/>
-      <c r="Q21" s="70">
-        <f>IF(J21&lt;=0,0,O21*State!$B$48/1000/J21)</f>
-        <v/>
-      </c>
-      <c r="R21" s="69" t="n"/>
-      <c r="T21" s="34" t="inlineStr">
-        <is>
-          <t>B.   Yes, every £1 returns £1.66</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="B22" s="24" t="inlineStr">
-        <is>
-          <t>Direct mail</t>
-        </is>
-      </c>
-      <c r="C22" s="69" t="n"/>
-      <c r="D22" s="69" t="n"/>
-      <c r="E22" s="69" t="n"/>
-      <c r="F22" s="69" t="n"/>
-      <c r="G22" s="25">
-        <f>State!$C$62</f>
-        <v/>
-      </c>
-      <c r="H22" s="69" t="n"/>
-      <c r="I22" s="69" t="n"/>
-      <c r="J22" s="26">
-        <f>IF(State!$B$64=1,State!$E$62,State!$B$62)</f>
-        <v/>
-      </c>
-      <c r="K22" s="69" t="n"/>
-      <c r="L22" s="69" t="n"/>
-      <c r="M22" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N22" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O22" s="28">
-        <f>IF(J22&lt;=0,0,(State!$D$62*State!$C$62*1000/90)/SQRT(State!$C$62)*SQRT(J22))</f>
-        <v/>
-      </c>
-      <c r="P22" s="69" t="n"/>
-      <c r="Q22" s="70">
-        <f>IF(J22&lt;=0,0,O22*State!$B$48/1000/J22)</f>
-        <v/>
-      </c>
-      <c r="R22" s="69" t="n"/>
-      <c r="T22" s="34" t="inlineStr">
-        <is>
-          <t>C.   No, cut everything</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="B23" s="24" t="inlineStr">
-        <is>
-          <t>Door drops</t>
-        </is>
-      </c>
-      <c r="C23" s="69" t="n"/>
-      <c r="D23" s="69" t="n"/>
-      <c r="E23" s="69" t="n"/>
-      <c r="F23" s="69" t="n"/>
-      <c r="G23" s="25">
-        <f>State!$C$63</f>
-        <v/>
-      </c>
-      <c r="H23" s="69" t="n"/>
-      <c r="I23" s="69" t="n"/>
-      <c r="J23" s="26">
-        <f>IF(State!$B$64=1,State!$E$63,State!$B$63)</f>
-        <v/>
-      </c>
-      <c r="K23" s="69" t="n"/>
-      <c r="L23" s="69" t="n"/>
-      <c r="M23" s="27" t="inlineStr">
-        <is>
-          <t>−</t>
-        </is>
-      </c>
-      <c r="N23" s="27" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="O23" s="28">
-        <f>IF(J23&lt;=0,0,(State!$D$63*State!$C$63*1000/90)/SQRT(State!$C$63)*SQRT(J23))</f>
-        <v/>
-      </c>
-      <c r="P23" s="69" t="n"/>
-      <c r="Q23" s="70">
-        <f>IF(J23&lt;=0,0,O23*State!$B$48/1000/J23)</f>
-        <v/>
-      </c>
-      <c r="R23" s="69" t="n"/>
-      <c r="T23" s="16">
-        <f>IF(State!$B$24=0,"Pick one.",IF(State!$B$24=State!$C$24,"✓ Moving money between channels was worth about £1.1m before adding a single pound.","✗ Not quite. The average pound looks great. The next pound does not."))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="B24" s="35" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="G24" s="36">
-        <f>SUM(G11:G23)</f>
-        <v/>
-      </c>
-      <c r="J24" s="37">
-        <f>SUM(J11:J23)</f>
-        <v/>
-      </c>
-      <c r="O24" s="36">
-        <f>SUM(O11:O23)</f>
-        <v/>
-      </c>
-      <c r="Q24" s="72">
-        <f>O24*State!$B$48/1000/J24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="T25" s="32">
-        <f>IF(LEFT(T23,1)="✓","Economists call this: Marginal return","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="B26" s="39" t="inlineStr">
-        <is>
-          <t>Each channel's curve is set so the 2025 plan gives exactly Wave 1's return. Double a channel's spend and you get 41% more sign-ups, not double. AP's real curves differ by channel, so their plan gained 12,300 sign-ups with them and about 600 here. The direction is the lesson.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1"/>
-    <row r="28" ht="10" customHeight="1"/>
-    <row r="29" ht="34" customHeight="1">
-      <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>◀  Back</t>
-        </is>
-      </c>
-      <c r="C29" s="67" t="n"/>
-      <c r="D29" s="67" t="n"/>
-      <c r="E29" s="68" t="n"/>
-      <c r="G29" s="19">
-        <f>IF(State!$B$64=1,"Back to my plan","Show AP's plan")</f>
-        <v/>
-      </c>
-      <c r="H29" s="67" t="n"/>
-      <c r="I29" s="67" t="n"/>
-      <c r="J29" s="68" t="n"/>
-      <c r="L29" s="19" t="inlineStr">
-        <is>
-          <t>Reset plan</t>
-        </is>
-      </c>
-      <c r="M29" s="67" t="n"/>
-      <c r="N29" s="67" t="n"/>
-      <c r="O29" s="68" t="n"/>
-      <c r="T29" s="21" t="inlineStr">
-        <is>
-          <t>Next  ▶</t>
-        </is>
-      </c>
-      <c r="U29" s="67" t="n"/>
-      <c r="V29" s="67" t="n"/>
-      <c r="W29" s="67" t="n"/>
-      <c r="X29" s="67" t="n"/>
-      <c r="Y29" s="67" t="n"/>
-      <c r="Z29" s="68" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="89">
-    <mergeCell ref="Q13:R13"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="T23:Z24"/>
-    <mergeCell ref="B26:R27"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q11:R11"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="T2:Z2"/>
-    <mergeCell ref="T18:Z19"/>
-    <mergeCell ref="N10"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="J24:L24"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="J16:L16"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="Q23:R23"/>
-    <mergeCell ref="T29:Z29"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B7:Z7"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="J14:L14"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="L29:O29"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="G22:I22"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="M10"/>
-    <mergeCell ref="J10:L10"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="O10:P10"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q24:R24"/>
-    <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="T13:Z15"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B5:Z5"/>
-    <mergeCell ref="J22:L22"/>
-    <mergeCell ref="Q10:R10"/>
-    <mergeCell ref="Q19:R19"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="J23:L23"/>
-    <mergeCell ref="Q22:R22"/>
-    <mergeCell ref="O12:P12"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="O13:P13"/>
-  </mergeCells>
-  <conditionalFormatting sqref="B3:Y3">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>COLUMN()-1&lt;=State!$B$31</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11:J23">
-    <cfRule type="dataBar" priority="2">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="1600"/>
-        <color rgb="00009CEE"/>
-      </dataBar>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T12">
-    <cfRule type="expression" priority="3" dxfId="9">
-      <formula>ISNUMBER(SEARCH("Good",T12))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="10">
-      <formula>NOT(ISNUMBER(SEARCH("Good",T12)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T13">
-    <cfRule type="expression" priority="5" dxfId="6">
-      <formula>LEFT(T13,1)="✓"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7">
-      <formula>LEFT(T13,1)&lt;&gt;"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T20">
-    <cfRule type="expression" priority="7" dxfId="4">
-      <formula>State!$B$24=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T21">
-    <cfRule type="expression" priority="8" dxfId="4">
-      <formula>State!$B$24=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T22">
-    <cfRule type="expression" priority="9" dxfId="4">
-      <formula>State!$B$24=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T23">
-    <cfRule type="expression" priority="10" dxfId="6">
-      <formula>LEFT(T23,1)="✓"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="7">
-      <formula>LEFT(T23,1)="✗"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LCRUK CONFIDENTIAL, INTERNAL USE ONLY</oddHeader>
-    <oddFooter>&amp;LThe Econometrics Game v3&amp;RAndrew Rajanathan, CRUK M&amp;&amp;D</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet3">
     <tabColor rgb="00009CEE"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -3359,7 +3138,7 @@
     <row r="1" ht="8" customHeight="1"/>
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="1">
-        <f>"Chapter 9  ·  The long game"</f>
+        <f>"Chapter 9  ·  Brand"</f>
         <v/>
       </c>
       <c r="T2" s="2">
@@ -3579,9 +3358,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet4">
+  <sheetPr codeName="Sheet3">
     <tabColor rgb="00009CEE"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -3928,9 +3707,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet5">
+  <sheetPr codeName="Sheet4">
     <tabColor rgb="001B2A4A"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
@@ -4257,9 +4036,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet6">
+  <sheetPr codeName="Sheet5">
     <tabColor rgb="00878787"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -4720,9 +4499,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet7">
+  <sheetPr codeName="Sheet6">
     <tabColor rgb="00878787"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -40082,13 +39861,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet8">
+  <sheetPr codeName="Sheet7">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41814,6 +41593,66 @@
         <v>6</v>
       </c>
       <c r="U22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>The next pound</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Where should the next pound go?</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Chapter 8 is the budget game, just below this screen. Scroll down if you cannot see it.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Tap − and + to move money between the thirteen 2025 channels. Keep the total. Beat the 2025 plan, then answer the question.</t>
+        </is>
+      </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" t="n">
+        <v>6</v>
+      </c>
+      <c r="U23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -41831,9 +41670,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Sheet9">
+  <sheetPr codeName="Sheet8">
     <tabColor rgb="00FFC000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -41856,7 +41695,7 @@
       </c>
       <c r="D1" s="60" t="inlineStr">
         <is>
-          <t>No macros? This tab is the control panel. Type the step number in B1 (1 to 21), the dials in B2 to B12, quiz answers in B17 to B26 and the budget in B51 to B63. Set B30 to 2, 3, 4 or 5 to move to the later chapters.</t>
+          <t>No macros? This tab is the control panel. Type the step number in B1 (1 to 22; step 22 is the budget game lower down the Race for Life tab), the dials in B2 to B12, quiz answers in B17 to B26 and the budget in B51 to B63. Set B30 to 2 (Brand), 3 (Giving) or 4 (Finish) to move on.</t>
         </is>
       </c>
     </row>
@@ -42150,7 +41989,7 @@
     <row r="30">
       <c r="A30" s="58" t="inlineStr">
         <is>
-          <t>Stage (1 Play, 2 Budget, 3 Long game, 4 Giving, 5 Finish)</t>
+          <t>Stage (1 Race for Life, 2 Brand, 3 Giving, 4 Finish)</t>
         </is>
       </c>
       <c r="B30" s="58" t="n">
@@ -42164,7 +42003,7 @@
         </is>
       </c>
       <c r="B31" s="58">
-        <f>IF(B30=1,B1,MIN(24,21+B30-1))</f>
+        <f>IF(B30=1,MIN(22,B1),MIN(24,22+B30-1))</f>
         <v/>
       </c>
     </row>
@@ -42179,7 +42018,7 @@
         </is>
       </c>
       <c r="B33" s="58">
-        <f>INDEX(Steps!$F$2:$F$22,State!$B$1)</f>
+        <f>INDEX(Steps!$F$2:$F$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42190,7 +42029,7 @@
         </is>
       </c>
       <c r="B34" s="58">
-        <f>INDEX(Steps!$G$2:$G$22,State!$B$1)</f>
+        <f>INDEX(Steps!$G$2:$G$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42201,7 +42040,7 @@
         </is>
       </c>
       <c r="B35" s="58">
-        <f>INDEX(Steps!$J$2:$J$22,State!$B$1)</f>
+        <f>INDEX(Steps!$J$2:$J$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42212,7 +42051,7 @@
         </is>
       </c>
       <c r="B36" s="58">
-        <f>INDEX(Steps!$K$2:$K$22,State!$B$1)</f>
+        <f>INDEX(Steps!$K$2:$K$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42234,7 +42073,7 @@
         </is>
       </c>
       <c r="B38" s="58">
-        <f>INDEX(Steps!$S$2:$S$22,State!$B$1)</f>
+        <f>INDEX(Steps!$S$2:$S$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42256,7 +42095,7 @@
         </is>
       </c>
       <c r="B40" s="58">
-        <f>INDEX(Steps!$R$2:$R$22,State!$B$1)</f>
+        <f>INDEX(Steps!$R$2:$R$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42289,7 +42128,7 @@
         </is>
       </c>
       <c r="B43" s="58">
-        <f>INDEX(Steps!$T$2:$T$22,State!$B$1)</f>
+        <f>INDEX(Steps!$T$2:$T$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42300,7 +42139,7 @@
         </is>
       </c>
       <c r="B44" s="58">
-        <f>INDEX(Steps!$U$2:$U$22,State!$B$1)</f>
+        <f>INDEX(Steps!$U$2:$U$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42311,7 +42150,7 @@
         </is>
       </c>
       <c r="B45" s="58">
-        <f>INDEX(Steps!$W$2:$W$22,State!$B$1)</f>
+        <f>INDEX(Steps!$W$2:$W$23,State!$B$1)</f>
         <v/>
       </c>
     </row>
@@ -42784,4 +42623,165 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Sheet9">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="50" t="inlineStr">
+        <is>
+          <t>Room notes: running the game with a team in 45 minutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="65" t="inlineStr">
+        <is>
+          <t>For the person leading. Unhide from the sheet list. The answers are here, so do not share the screen with this tab open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="B5" s="66" t="inlineStr">
+        <is>
+          <t>0 to 5</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Open the Race for Life tab on the big screen. Chapter 1, one person tapping. Ask the room what made the spikes before anyone taps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="B6" s="66" t="inlineStr">
+        <is>
+          <t>5 to 15</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Chapters 2 and 3 together. Ask for a show of hands before each number: higher or lower than a thousand? The base surprises people. Let it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="B7" s="66" t="inlineStr">
+        <is>
+          <t>15 to 25</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Chapter 4. Ask the room to guess the memory before you touch it. Most say 20%. Show what 80% does. Name adstock only after the line fits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>25 to 32</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Chapter 5. Add the halo, then read the 42% step out loud and stop. Let the room say what it means for next year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="B9" s="66" t="inlineStr">
+        <is>
+          <t>32 to 38</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>Chapter 6 in pairs on laptops. The point is the catch, not the numbers. Ask: which channel are you least sure of, and why?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="B10" s="66" t="inlineStr">
+        <is>
+          <t>38 to 45</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Chapter 8 as a race: first to 1,000 extra sign-ups on the same money. Close on average versus last pound. The Brand and Giving tabs are homework.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="49" customHeight="1">
+      <c r="B11" s="66" t="inlineStr">
+        <is>
+          <t>Answer key</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Base 876. Brake 952. Sale 7,598. Adverts 16.1 per £1,000, memory 80%. Halo 2.86 per £1,000. Channels: TV 17.0, Online video 17.4, Radio 17.4, Posters 6.1, Digital and social 17.6. Every quiz answer is A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="49" customHeight="1">
+      <c r="B12" s="66" t="inlineStr">
+        <is>
+          <t>If asked "is this just correlation?"</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>Partly, and AP say so. Three things make it more: it controls for everything at once, it is tested on weeks it never saw, and channels that stopped (Race for Life TV after 2024) let it see what happens without them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="B13" s="66" t="inlineStr">
+        <is>
+          <t>If asked "the halo felt too big"</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>It did, and AP rebuilt it. They now measure Committed Giving as one block. The halo fell and is still 5% of 2025 sign-ups and 9,139 of the 2025 decline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="B14" s="66" t="inlineStr">
+        <is>
+          <t>Budget chapter</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>Best possible on the game's curves is about 2,000 extra: cut posters and telemarketing, add DRTV and online video. AP's own plan shows the same direction.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9"/>
+  <headerFooter>
+    <oddHeader>&amp;LCRUK CONFIDENTIAL, INTERNAL USE ONLY</oddHeader>
+    <oddFooter>&amp;LThe Econometrics Game v3&amp;RAndrew Rajanathan, CRUK M&amp;&amp;D</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tighten claims against the Wave 1 sources
Label fitted answers as fitted rather than as Wave 1 numbers, note
emails inside the base and AP's near-zero baseline, correct the driver
count, rename the fifth channel group, and reword the Committed Giving
return to what AP measured.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DFB7finRRwjLofP9hApkAo
</commit_message>
<xml_diff>
--- a/econometrics-game/CRUK_Econometrics_Game_v3_no_macros.xlsx
+++ b/econometrics-game/CRUK_Econometrics_Game_v3_no_macros.xlsx
@@ -1747,7 +1747,7 @@
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="T15" s="8">
-        <f>IF(State!$B$33="quiz","C.   "&amp;INDEX(Steps!$Q$2:$Q$23,State!$B$1),IF(State!$B$33="dials5","Digital and social:  "&amp;TEXT(State!$B$12,"0.0")&amp;" per £1,000",""))</f>
+        <f>IF(State!$B$33="quiz","C.   "&amp;INDEX(Steps!$Q$2:$Q$23,State!$B$1),IF(State!$B$33="dials5","Digital, social and the rest:  "&amp;TEXT(State!$B$12,"0.0")&amp;" per £1,000",""))</f>
         <v/>
       </c>
       <c r="U15" s="9">
@@ -1812,7 +1812,7 @@
     <row r="26" ht="26" customHeight="1"/>
     <row r="27" ht="24" customHeight="1">
       <c r="T27" s="18">
-        <f>IF(State!$B$14=1,IF(State!$B$33="dial","Wave 1's number: "&amp;TEXT(State!$B$35,State!$B$45),IF(State!$B$33="dials5","Wave 1: "&amp;TEXT(Answers!E16,"0.0")&amp;", "&amp;TEXT(Answers!E17,"0.0")&amp;", "&amp;TEXT(Answers!E18,"0.0")&amp;", "&amp;TEXT(Answers!E19,"0.0")&amp;", "&amp;TEXT(Answers!E20,"0.0"),IF(State!$B$33="quiz","Wave 1's answer: "&amp;CHOOSE(State!$B$40,"A","B","C"),"Wave 1's model is the grey dashed line."))),"")</f>
+        <f>IF(State!$B$14=1,IF(State!$B$33="dial","Answer, fitted to Wave 1: "&amp;TEXT(State!$B$35,State!$B$45),IF(State!$B$33="dials5","Fitted to Wave 1: "&amp;TEXT(Answers!E16,"0.0")&amp;", "&amp;TEXT(Answers!E17,"0.0")&amp;", "&amp;TEXT(Answers!E18,"0.0")&amp;", "&amp;TEXT(Answers!E19,"0.0")&amp;", "&amp;TEXT(Answers!E20,"0.0"),IF(State!$B$33="quiz","Wave 1's answer: "&amp;CHOOSE(State!$B$40,"A","B","C"),"Wave 1's model is the grey dashed line."))),"")</f>
         <v/>
       </c>
     </row>
@@ -3067,7 +3067,7 @@
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>Digital and social: memory %</t>
+          <t>Digital, social and the rest: memory %</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Digital and social: sign-ups per £1,000</t>
+          <t>Digital, social and the rest: sign-ups per £1,000</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -3439,7 +3439,7 @@
     <row r="4" ht="8" customHeight="1"/>
     <row r="5" ht="40" customHeight="1">
       <c r="B5" s="4">
-        <f>"Committed Giving looks like 9p per £1 because the model only counts the first gift"</f>
+        <f>"Committed Giving looks like 9p per £1 because the model only counts new givers inside the window"</f>
         <v/>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
     <row r="17" ht="34" customHeight="1">
       <c r="T17" s="41" t="inlineStr">
         <is>
-          <t>counts only the first gift of brand new givers. Not the years that follow, not the churn adverts prevent.</t>
+          <t>counts only the income from brand new givers inside the modelled window, about £300 each. Not the existing book, not the years that follow, not the churn adverts prevent.</t>
         </is>
       </c>
       <c r="AC17" s="42" t="inlineStr">
@@ -3598,7 +3598,7 @@
     <row r="20" ht="24" customHeight="1">
       <c r="T20" s="34" t="inlineStr">
         <is>
-          <t>A.   It counts only the first gift of new givers</t>
+          <t>A.   It counts only new givers, inside the modelled window</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="G27" s="31" t="inlineStr">
         <is>
-          <t>Committed Giving shows 9p per pound because the model only counts the first gift of brand new givers.</t>
+          <t>Committed Giving shows 9p per pound because the model only counts new givers inside the modelled window, not the years of giving that follow.</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="D8" s="49" t="inlineStr">
         <is>
-          <t>AP tested 18 marketing drivers and six others and kept those with a reliable link. Weather, PR and outages had none.</t>
+          <t>AP tested 18 marketing drivers and seven others and kept those with a reliable link. Weather, PR and outages had none.</t>
         </is>
       </c>
       <c r="E8" s="49" t="inlineStr">
@@ -4668,7 +4668,7 @@
       </c>
       <c r="R5" s="47" t="inlineStr">
         <is>
-          <t>Digital and social £k</t>
+          <t>Digital, social and the rest £k</t>
         </is>
       </c>
       <c r="S5" s="47" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="AI5" s="47" t="inlineStr">
         <is>
-          <t>Your block: Digital and social</t>
+          <t>Your block: Digital, social and the rest</t>
         </is>
       </c>
       <c r="AJ5" s="47" t="inlineStr">
@@ -4828,7 +4828,7 @@
       </c>
       <c r="BB5" s="47" t="inlineStr">
         <is>
-          <t>AP block: Digital and social</t>
+          <t>AP block: Digital, social and the rest</t>
         </is>
       </c>
       <c r="BC5" s="47" t="inlineStr">
@@ -40243,7 +40243,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>About 900 a week sign up whatever we do. People who already know us, and the ones we email.</t>
+          <t>About 900 a week: people who already consider us, plus the ones we email. AP count emails as our own media, so this block is the base plus emails.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -40323,7 +40323,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Right. The base is small. Almost every other sign-up was caused by something we did.</t>
+          <t>Right, and once price and the shut window are counted AP put the true base close to zero. Almost every sign-up was caused by something we did.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -40804,7 +40804,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Memory of 80%: the effect fades slowly over months. Judge a campaign in week one and you miss most of it.</t>
+          <t>Memory of 80%: the effect fades slowly over months. AP do not publish the rate; this one is fitted to their weekly line. Judge a campaign in week one and you miss most of it.</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -41175,7 +41175,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>TV, video, radio, posters, digital. They mostly run in the same weeks. Tap − and + on each until all five ticks show.</t>
+          <t>TV, video, radio, posters, and digital, social and the rest. They mostly run in the same weeks. Tap − and + on each until all five ticks show.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -41360,7 +41360,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Digital and social</t>
+          <t>Digital, social and the rest</t>
         </is>
       </c>
       <c r="R19" t="n">
@@ -42732,7 +42732,7 @@
       </c>
       <c r="C11" s="41" t="inlineStr">
         <is>
-          <t>Base 876. Brake 952. Sale 7,598. Adverts 16.1 per £1,000, memory 80%. Halo 2.86 per £1,000. Channels: TV 17.0, Online video 17.4, Radio 17.4, Posters 6.1, Digital and social 17.6. Every quiz answer is A.</t>
+          <t>Base 876. Brake 952. Sale 7,598. Adverts 16.1 per £1,000, memory 80%. Halo 2.86 per £1,000. Channels: TV 17.0, Online video 17.4, Radio 17.4, Posters 6.1, Digital, social and the rest 17.6. Every quiz answer is A.</t>
         </is>
       </c>
     </row>

</xml_diff>